<commit_message>
build: improve build process and repository cleanup
- Add Python syntax check before PyInstaller compilation.
- Enable optional custom icon support in build scripts.
- Expand .gitignore to exclude build artifacts, logs, and sensitive data.
- Update documentation and build process for cleaner distribution.
</commit_message>
<xml_diff>
--- a/event_list.xlsx
+++ b/event_list.xlsx
@@ -399,9 +399,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C2"/>
   <cols>
-    <col min="1" max="1" width="38.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="28.83203125" customWidth="1"/>
+    <col min="1" max="1" width="35.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -417,10 +417,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Солодовникова Романа Александровна</v>
+        <v>Иванов Иван Иванович</v>
       </c>
       <c r="B2" t="str">
-        <v>23.06.2005</v>
+        <v>15.05.2012</v>
       </c>
       <c r="C2" t="str">
         <v/>

</xml_diff>